<commit_message>
<= max_row, not <
</commit_message>
<xml_diff>
--- a/tests/wson-test.xlsx
+++ b/tests/wson-test.xlsx
@@ -5,11 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="FullTest" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="TopLevelArray" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="56">
   <si>
     <t xml:space="preserve">&gt;</t>
   </si>
@@ -186,6 +187,9 @@
   </si>
   <si>
     <t xml:space="preserve">charlie@example.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test</t>
   </si>
 </sst>
 </file>
@@ -952,4 +956,34 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="B2:D2"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: parsing in parseArray/parseObject
</commit_message>
<xml_diff>
--- a/tests/wson-test.xlsx
+++ b/tests/wson-test.xlsx
@@ -341,7 +341,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -374,15 +374,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -411,7 +407,6 @@
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </dxf>
   </dxfs>
   <colors>
@@ -657,7 +652,7 @@
   <dimension ref="B2:K22"/>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="4.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14.93"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.77"/>
@@ -863,7 +858,7 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="7" t="s">
         <v>45</v>
       </c>
       <c r="D21" s="1" t="s">
@@ -871,7 +866,7 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="7" t="s">
         <v>47</v>
       </c>
       <c r="D22" s="1" t="s">
@@ -932,7 +927,7 @@
       <c r="C5" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="8" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -969,7 +964,7 @@
       <c r="C10" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="8" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -1006,7 +1001,7 @@
       <c r="C15" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="D15" s="8" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1032,17 +1027,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:D2"/>
+  <dimension ref="B1:D2"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="0" t="s">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1062,28 +1058,29 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:D3"/>
+  <dimension ref="B1:D3"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="9" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1108,25 +1105,26 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:D3"/>
+  <dimension ref="B1:D3"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="0" t="s">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C3" s="0" t="s">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>38</v>
       </c>
     </row>

</xml_diff>